<commit_message>
Broaden legal SMB coverage
</commit_message>
<xml_diff>
--- a/exports/complycheck_nis2_vendor_catalog_v5.xlsx
+++ b/exports/complycheck_nis2_vendor_catalog_v5.xlsx
@@ -923,7 +923,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1079,7 +1079,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2639,7 +2639,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3731,7 +3731,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3887,7 +3887,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4043,7 +4043,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4979,7 +4979,7 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5291,7 +5291,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -5603,7 +5603,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -5915,7 +5915,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -6227,7 +6227,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -7163,7 +7163,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -14894,7 +14894,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -15198,7 +15198,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -15350,7 +15350,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -15502,7 +15502,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -16110,7 +16110,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -16414,7 +16414,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -16566,7 +16566,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -16718,7 +16718,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -17022,7 +17022,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -17326,7 +17326,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -17630,7 +17630,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -17782,7 +17782,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -17934,7 +17934,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -18086,7 +18086,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -18390,7 +18390,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -18542,7 +18542,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -18998,7 +18998,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -19150,7 +19150,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -19454,7 +19454,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mindre og mellemstore virksomheder</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mindre og mellemstore virksomheder</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -19606,7 +19606,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -19758,7 +19758,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -20062,7 +20062,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -20214,7 +20214,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -20366,7 +20366,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -20518,7 +20518,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -20670,7 +20670,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -20822,7 +20822,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -20974,7 +20974,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -21126,7 +21126,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -21278,7 +21278,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -21430,7 +21430,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -21734,7 +21734,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -21886,7 +21886,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -22038,7 +22038,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -22190,7 +22190,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -22342,7 +22342,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -22494,7 +22494,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -22646,7 +22646,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -22798,7 +22798,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -36030,7 +36030,7 @@
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="82" customWidth="1" min="8" max="8"/>
@@ -36433,7 +36433,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -36589,7 +36589,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -38149,7 +38149,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -39241,7 +39241,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -39397,7 +39397,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -39553,7 +39553,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -40489,7 +40489,7 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -40801,7 +40801,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -41113,7 +41113,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -41425,7 +41425,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -41737,7 +41737,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market, enterprise</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -42673,7 +42673,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mid-market, enterprise</t>
+          <t>SMB, mid-market</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -50896,7 +50896,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -51048,7 +51048,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -51200,7 +51200,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -51352,7 +51352,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -51504,7 +51504,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -51656,7 +51656,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -51808,7 +51808,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -51960,7 +51960,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -52112,7 +52112,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -52264,7 +52264,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -52416,7 +52416,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -52568,7 +52568,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -52720,7 +52720,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -52872,7 +52872,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -53024,7 +53024,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -53328,7 +53328,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -53480,7 +53480,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -53632,7 +53632,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -53784,7 +53784,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -53936,7 +53936,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -54088,7 +54088,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -54392,7 +54392,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -54544,7 +54544,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -54696,7 +54696,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -54848,7 +54848,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -55000,7 +55000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -55152,7 +55152,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -55304,7 +55304,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -55456,7 +55456,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mindre og mellemstore virksomheder</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mindre og mellemstore virksomheder</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -55608,7 +55608,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, inklusive netværkssikkerhed, segmentering og hardening, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -55760,7 +55760,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, samt backup, recovery og robust it-drift, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -56064,7 +56064,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -56216,7 +56216,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -56368,7 +56368,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -56520,7 +56520,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -56672,7 +56672,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, fra mindre virksomheder til større enterprise-miljøer</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -56824,7 +56824,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -56976,7 +56976,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -57128,7 +57128,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -57280,7 +57280,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -57432,7 +57432,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -57584,7 +57584,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -57736,7 +57736,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -57888,7 +57888,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -58040,7 +58040,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -58192,7 +58192,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -58344,7 +58344,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -58496,7 +58496,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med tydelig cloud- og platformskompetence, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, med tydelig cloud- og platformskompetence, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -58648,7 +58648,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -58800,7 +58800,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, primært til mellemstore og større organisationer</t>
+          <t>Teknisk implementering af sikkerhedskontroller, arkitektur, adgangsstyring, logging og driftsnære forbedringer, med fokus på identitet, adgangsstyring og privilegerede konti, primært til mellemstore og større organisationer</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">

</xml_diff>